<commit_message>
feat: :zap: se agregaron detallles
se agregaron detalles y se solucionaron errores basicos
</commit_message>
<xml_diff>
--- a/reportes/movimientos.xlsx
+++ b/reportes/movimientos.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -427,51 +427,51 @@
     </row>
     <row r="2">
       <c r="A2">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-06-12 07:19:19</v>
+        <v>2026-06-13 20:18:04</v>
       </c>
       <c r="C2" t="str">
-        <v>entrada</v>
+        <v>venta</v>
       </c>
       <c r="D2" t="str">
-        <v>Pantalon</v>
+        <v>Bata Azul</v>
       </c>
       <c r="E2" t="str">
-        <v>10-12</v>
+        <v>Unica</v>
       </c>
       <c r="F2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G2" t="str">
         <v>Administrador</v>
       </c>
       <c r="H2" t="str">
-        <v>Entrada de stock</v>
+        <v>Venta registrada</v>
       </c>
     </row>
     <row r="3">
       <c r="A3">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B3" t="str">
-        <v>2026-06-12 06:44:32</v>
+        <v>2026-06-12 07:19:19</v>
       </c>
       <c r="C3" t="str">
         <v>entrada</v>
       </c>
       <c r="D3" t="str">
-        <v>Camisa Gala</v>
+        <v>Pantalon</v>
       </c>
       <c r="E3" t="str">
-        <v>M-L</v>
+        <v>10-12</v>
       </c>
       <c r="F3">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G3" t="str">
-        <v>achinti morales hernández</v>
+        <v>Administrador</v>
       </c>
       <c r="H3" t="str">
         <v>Entrada de stock</v>
@@ -479,36 +479,36 @@
     </row>
     <row r="4">
       <c r="A4">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B4" t="str">
-        <v>2026-06-12 06:36:20</v>
+        <v>2026-06-12 06:44:32</v>
       </c>
       <c r="C4" t="str">
-        <v>venta</v>
+        <v>entrada</v>
       </c>
       <c r="D4" t="str">
-        <v>Pantalon</v>
+        <v>Camisa Gala</v>
       </c>
       <c r="E4" t="str">
-        <v>10-12</v>
+        <v>M-L</v>
       </c>
       <c r="F4">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G4" t="str">
-        <v>Administrador</v>
+        <v>achinti morales hernández</v>
       </c>
       <c r="H4" t="str">
-        <v>Venta registrada</v>
+        <v>Entrada de stock</v>
       </c>
     </row>
     <row r="5">
       <c r="A5">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B5" t="str">
-        <v>2026-06-12 06:31:22</v>
+        <v>2026-06-12 06:36:20</v>
       </c>
       <c r="C5" t="str">
         <v>venta</v>
@@ -526,12 +526,38 @@
         <v>Administrador</v>
       </c>
       <c r="H5" t="str">
+        <v>Venta registrada</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <v>33</v>
+      </c>
+      <c r="B6" t="str">
+        <v>2026-06-12 06:31:22</v>
+      </c>
+      <c r="C6" t="str">
+        <v>venta</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Pantalon</v>
+      </c>
+      <c r="E6" t="str">
+        <v>10-12</v>
+      </c>
+      <c r="F6">
+        <v>1</v>
+      </c>
+      <c r="G6" t="str">
+        <v>Administrador</v>
+      </c>
+      <c r="H6" t="str">
         <v>Venta registrada</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: :bug: repare errores que habia antes de la entrega del programa
</commit_message>
<xml_diff>
--- a/reportes/movimientos.xlsx
+++ b/reportes/movimientos.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H20"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -427,39 +427,39 @@
     </row>
     <row r="2">
       <c r="A2">
-        <v>37</v>
+        <v>51</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-06-13 20:18:04</v>
+        <v>2026-06-17 07:39:58</v>
       </c>
       <c r="C2" t="str">
-        <v>venta</v>
+        <v>entrada</v>
       </c>
       <c r="D2" t="str">
-        <v>Bata Azul</v>
+        <v>Pantalon</v>
       </c>
       <c r="E2" t="str">
-        <v>Unica</v>
+        <v>10-12</v>
       </c>
       <c r="F2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G2" t="str">
-        <v>Administrador</v>
+        <v>achinti morales hernández</v>
       </c>
       <c r="H2" t="str">
-        <v>Venta registrada</v>
+        <v>Entrada de stock</v>
       </c>
     </row>
     <row r="3">
       <c r="A3">
-        <v>36</v>
+        <v>50</v>
       </c>
       <c r="B3" t="str">
-        <v>2026-06-12 07:19:19</v>
+        <v>2026-06-16 20:39:32</v>
       </c>
       <c r="C3" t="str">
-        <v>entrada</v>
+        <v>venta</v>
       </c>
       <c r="D3" t="str">
         <v>Pantalon</v>
@@ -468,50 +468,50 @@
         <v>10-12</v>
       </c>
       <c r="F3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G3" t="str">
-        <v>Administrador</v>
+        <v>achinti morales hernández</v>
       </c>
       <c r="H3" t="str">
-        <v>Entrada de stock</v>
+        <v>Venta registrada</v>
       </c>
     </row>
     <row r="4">
       <c r="A4">
-        <v>35</v>
+        <v>49</v>
       </c>
       <c r="B4" t="str">
-        <v>2026-06-12 06:44:32</v>
+        <v>2026-06-16 20:39:20</v>
       </c>
       <c r="C4" t="str">
-        <v>entrada</v>
+        <v>venta</v>
       </c>
       <c r="D4" t="str">
-        <v>Camisa Gala</v>
+        <v>Pantalon</v>
       </c>
       <c r="E4" t="str">
-        <v>M-L</v>
+        <v>10-12</v>
       </c>
       <c r="F4">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G4" t="str">
         <v>achinti morales hernández</v>
       </c>
       <c r="H4" t="str">
-        <v>Entrada de stock</v>
+        <v>Venta registrada</v>
       </c>
     </row>
     <row r="5">
       <c r="A5">
-        <v>34</v>
+        <v>48</v>
       </c>
       <c r="B5" t="str">
-        <v>2026-06-12 06:36:20</v>
+        <v>2026-06-16 19:42:36</v>
       </c>
       <c r="C5" t="str">
-        <v>venta</v>
+        <v>entrada</v>
       </c>
       <c r="D5" t="str">
         <v>Pantalon</v>
@@ -520,44 +520,408 @@
         <v>10-12</v>
       </c>
       <c r="F5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G5" t="str">
-        <v>Administrador</v>
+        <v>achinti morales hernández</v>
       </c>
       <c r="H5" t="str">
-        <v>Venta registrada</v>
+        <v>Entrada de stock</v>
       </c>
     </row>
     <row r="6">
       <c r="A6">
+        <v>47</v>
+      </c>
+      <c r="B6" t="str">
+        <v>2026-06-16 19:42:27</v>
+      </c>
+      <c r="C6" t="str">
+        <v>entrada</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Bata Azul</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Unica</v>
+      </c>
+      <c r="F6">
+        <v>2</v>
+      </c>
+      <c r="G6" t="str">
+        <v>achinti morales hernández</v>
+      </c>
+      <c r="H6" t="str">
+        <v>Entrada de stock</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <v>46</v>
+      </c>
+      <c r="B7" t="str">
+        <v>2026-06-16 16:32:55</v>
+      </c>
+      <c r="C7" t="str">
+        <v>venta</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Bata Manga Larga</v>
+      </c>
+      <c r="E7" t="str">
+        <v>M-L</v>
+      </c>
+      <c r="F7">
+        <v>1</v>
+      </c>
+      <c r="G7" t="str">
+        <v>achinti morales hernández</v>
+      </c>
+      <c r="H7" t="str">
+        <v>Venta registrada</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <v>43</v>
+      </c>
+      <c r="B8" t="str">
+        <v>2026-06-16 16:22:12</v>
+      </c>
+      <c r="C8" t="str">
+        <v>venta</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Buso</v>
+      </c>
+      <c r="E8" t="str">
+        <v>XS-S</v>
+      </c>
+      <c r="F8">
+        <v>1</v>
+      </c>
+      <c r="G8" t="str">
+        <v>achinti morales hernández</v>
+      </c>
+      <c r="H8" t="str">
+        <v>Venta registrada</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <v>44</v>
+      </c>
+      <c r="B9" t="str">
+        <v>2026-06-16 16:22:12</v>
+      </c>
+      <c r="C9" t="str">
+        <v>venta</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Buso</v>
+      </c>
+      <c r="E9" t="str">
+        <v>L-XL</v>
+      </c>
+      <c r="F9">
+        <v>1</v>
+      </c>
+      <c r="G9" t="str">
+        <v>achinti morales hernández</v>
+      </c>
+      <c r="H9" t="str">
+        <v>Venta registrada</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10">
+        <v>45</v>
+      </c>
+      <c r="B10" t="str">
+        <v>2026-06-16 16:22:12</v>
+      </c>
+      <c r="C10" t="str">
+        <v>venta</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Guayabera Diario</v>
+      </c>
+      <c r="E10" t="str">
+        <v>M-L</v>
+      </c>
+      <c r="F10">
+        <v>1</v>
+      </c>
+      <c r="G10" t="str">
+        <v>achinti morales hernández</v>
+      </c>
+      <c r="H10" t="str">
+        <v>Venta registrada</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11">
+        <v>40</v>
+      </c>
+      <c r="B11" t="str">
+        <v>2026-06-16 14:29:33</v>
+      </c>
+      <c r="C11" t="str">
+        <v>venta</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Bata Azul</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Unica</v>
+      </c>
+      <c r="F11">
+        <v>1</v>
+      </c>
+      <c r="G11" t="str">
+        <v>achinti morales hernández</v>
+      </c>
+      <c r="H11" t="str">
+        <v>Venta registrada</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12">
+        <v>41</v>
+      </c>
+      <c r="B12" t="str">
+        <v>2026-06-16 14:29:33</v>
+      </c>
+      <c r="C12" t="str">
+        <v>venta</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Bermuda</v>
+      </c>
+      <c r="E12" t="str">
+        <v>12-14</v>
+      </c>
+      <c r="F12">
+        <v>1</v>
+      </c>
+      <c r="G12" t="str">
+        <v>achinti morales hernández</v>
+      </c>
+      <c r="H12" t="str">
+        <v>Venta registrada</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13">
+        <v>42</v>
+      </c>
+      <c r="B13" t="str">
+        <v>2026-06-16 14:29:33</v>
+      </c>
+      <c r="C13" t="str">
+        <v>venta</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Buso</v>
+      </c>
+      <c r="E13" t="str">
+        <v>12-14</v>
+      </c>
+      <c r="F13">
+        <v>1</v>
+      </c>
+      <c r="G13" t="str">
+        <v>achinti morales hernández</v>
+      </c>
+      <c r="H13" t="str">
+        <v>Venta registrada</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14">
+        <v>39</v>
+      </c>
+      <c r="B14" t="str">
+        <v>2026-06-16 06:31:39</v>
+      </c>
+      <c r="C14" t="str">
+        <v>venta</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Pantalon</v>
+      </c>
+      <c r="E14" t="str">
+        <v>10-12</v>
+      </c>
+      <c r="F14">
+        <v>1</v>
+      </c>
+      <c r="G14" t="str">
+        <v>achinti morales hernández</v>
+      </c>
+      <c r="H14" t="str">
+        <v>Venta registrada</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15">
+        <v>38</v>
+      </c>
+      <c r="B15" t="str">
+        <v>2026-06-16 06:30:06</v>
+      </c>
+      <c r="C15" t="str">
+        <v>venta</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Pantalon</v>
+      </c>
+      <c r="E15" t="str">
+        <v>10-12</v>
+      </c>
+      <c r="F15">
+        <v>1</v>
+      </c>
+      <c r="G15" t="str">
+        <v>achinti morales hernández</v>
+      </c>
+      <c r="H15" t="str">
+        <v>Venta registrada</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16">
+        <v>37</v>
+      </c>
+      <c r="B16" t="str">
+        <v>2026-06-13 20:18:04</v>
+      </c>
+      <c r="C16" t="str">
+        <v>venta</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Bata Azul</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Unica</v>
+      </c>
+      <c r="F16">
+        <v>1</v>
+      </c>
+      <c r="G16" t="str">
+        <v>Administrador</v>
+      </c>
+      <c r="H16" t="str">
+        <v>Venta registrada</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17">
+        <v>36</v>
+      </c>
+      <c r="B17" t="str">
+        <v>2026-06-12 07:19:19</v>
+      </c>
+      <c r="C17" t="str">
+        <v>entrada</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Pantalon</v>
+      </c>
+      <c r="E17" t="str">
+        <v>10-12</v>
+      </c>
+      <c r="F17">
+        <v>2</v>
+      </c>
+      <c r="G17" t="str">
+        <v>Administrador</v>
+      </c>
+      <c r="H17" t="str">
+        <v>Entrada de stock</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18">
+        <v>35</v>
+      </c>
+      <c r="B18" t="str">
+        <v>2026-06-12 06:44:32</v>
+      </c>
+      <c r="C18" t="str">
+        <v>entrada</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Camisa Gala</v>
+      </c>
+      <c r="E18" t="str">
+        <v>M-L</v>
+      </c>
+      <c r="F18">
+        <v>5</v>
+      </c>
+      <c r="G18" t="str">
+        <v>achinti morales hernández</v>
+      </c>
+      <c r="H18" t="str">
+        <v>Entrada de stock</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19">
+        <v>34</v>
+      </c>
+      <c r="B19" t="str">
+        <v>2026-06-12 06:36:20</v>
+      </c>
+      <c r="C19" t="str">
+        <v>venta</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Pantalon</v>
+      </c>
+      <c r="E19" t="str">
+        <v>10-12</v>
+      </c>
+      <c r="F19">
+        <v>1</v>
+      </c>
+      <c r="G19" t="str">
+        <v>Administrador</v>
+      </c>
+      <c r="H19" t="str">
+        <v>Venta registrada</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20">
         <v>33</v>
       </c>
-      <c r="B6" t="str">
+      <c r="B20" t="str">
         <v>2026-06-12 06:31:22</v>
       </c>
-      <c r="C6" t="str">
-        <v>venta</v>
-      </c>
-      <c r="D6" t="str">
+      <c r="C20" t="str">
+        <v>venta</v>
+      </c>
+      <c r="D20" t="str">
         <v>Pantalon</v>
       </c>
-      <c r="E6" t="str">
+      <c r="E20" t="str">
         <v>10-12</v>
       </c>
-      <c r="F6">
-        <v>1</v>
-      </c>
-      <c r="G6" t="str">
+      <c r="F20">
+        <v>1</v>
+      </c>
+      <c r="G20" t="str">
         <v>Administrador</v>
       </c>
-      <c r="H6" t="str">
+      <c r="H20" t="str">
         <v>Venta registrada</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H20"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>